<commit_message>
KFSPTS-38115: code review changes
</commit_message>
<xml_diff>
--- a/src/main/resources/edu/cornell/kfs/cemi/pdp/batch/Payment_Election.xlsx
+++ b/src/main/resources/edu/cornell/kfs/cemi/pdp/batch/Payment_Election.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://huroncg-my.sharepoint.com/personal/nalder_huronconsultinggroup_com/Documents/Documents/Clover DX/Final Templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nkk4/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="211" documentId="8_{EE36FCEF-48C1-47BF-9020-F5E10495F737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE3CFFE6-919B-4898-A258-670E3F8447F6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0B4E06-F29A-6F45-A2AA-F1805FD028CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15390" tabRatio="756" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35640" yWindow="1140" windowWidth="36400" windowHeight="20460" tabRatio="756" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Usage Notes" sheetId="3" state="hidden" r:id="rId1"/>
@@ -1691,10 +1691,9 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color indexed="8"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
           </rPr>
           <t>Role ID Reference will identify for whom the payment election is created for as well as what role. The ID consists of a type attribute, which should be set to "Employee_ID", "Contingent_Worker_ID", or "Student_ID", and a value attribute, such as "04345”.</t>
         </r>
@@ -6511,7 +6510,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="308">
   <si>
     <t>Element</t>
   </si>
@@ -7162,21 +7161,9 @@
     <t>CDXTest-01</t>
   </si>
   <si>
-    <t>Clover</t>
-  </si>
-  <si>
-    <t>USA_Payroll_Payment</t>
-  </si>
-  <si>
     <t>DIRECT_DEPOSIT</t>
   </si>
   <si>
-    <t>Payment 1</t>
-  </si>
-  <si>
-    <t>Clover Payment 1</t>
-  </si>
-  <si>
     <t>DDA</t>
   </si>
   <si>
@@ -7186,27 +7173,12 @@
     <t>011002343</t>
   </si>
   <si>
-    <t>Payment 2</t>
-  </si>
-  <si>
-    <t>Clover Payment 2</t>
-  </si>
-  <si>
-    <t>Payment 3</t>
-  </si>
-  <si>
-    <t>Clover Payment 3</t>
-  </si>
-  <si>
     <t>SA</t>
   </si>
   <si>
     <t>054001204</t>
   </si>
   <si>
-    <t>Scope: Current Active Payment elections for all converted employees (Group One tab will only include payroll payment elections)</t>
-  </si>
-  <si>
     <t>Submit Payment Election Enrollment: Group Two</t>
   </si>
   <si>
@@ -7291,26 +7263,7 @@
     <t>Distribution_Balance_2_1</t>
   </si>
   <si>
-    <t>Bonus</t>
-  </si>
-  <si>
-    <t>Expense_Payments</t>
-  </si>
-  <si>
-    <t>Bonus 1</t>
-  </si>
-  <si>
-    <t>Clover Bonus 1</t>
-  </si>
-  <si>
     <t>CDXTest-02</t>
-  </si>
-  <si>
-    <t>Scope: Current Active Payment elections for expenses</t>
-  </si>
-  <si>
-    <t>Ithaca - AP should provide data for expense payments.  (Nick/Jason to check with Jeff Stulgis)
-WCM - defaulted from the main bank account.  Only one account will be listed here.</t>
   </si>
   <si>
     <t>Submit Payment Election Enrollment: Group Three</t>
@@ -7500,7 +7453,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -7564,7 +7517,12 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -7688,9 +7646,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -7728,7 +7686,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -7834,7 +7792,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -7976,7 +7934,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -7985,14 +7943,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD5E9411-4886-4443-B735-F794B16E117C}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="97.85546875" customWidth="1"/>
-    <col min="3" max="3" width="106.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="28.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.83203125" customWidth="1"/>
+    <col min="3" max="3" width="106.5" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -8001,7 +7959,7 @@
       </c>
       <c r="C1"/>
     </row>
-    <row r="2" spans="1:3" ht="57.95">
+    <row r="2" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
@@ -8010,7 +7968,7 @@
       </c>
       <c r="C2"/>
     </row>
-    <row r="3" spans="1:3" ht="57.95">
+    <row r="3" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
         <v>4</v>
       </c>
@@ -8019,7 +7977,7 @@
       </c>
       <c r="C3"/>
     </row>
-    <row r="4" spans="1:3" ht="29.1">
+    <row r="4" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>6</v>
       </c>
@@ -8028,7 +7986,7 @@
       </c>
       <c r="C4"/>
     </row>
-    <row r="5" spans="1:3" ht="29.1">
+    <row r="5" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>8</v>
       </c>
@@ -8037,7 +7995,7 @@
       </c>
       <c r="C5"/>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>10</v>
       </c>
@@ -8046,15 +8004,15 @@
       </c>
       <c r="C6"/>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B7" s="1"/>
       <c r="C7"/>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B8" s="1"/>
       <c r="C8"/>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B9" s="1"/>
       <c r="C9"/>
     </row>
@@ -8065,141 +8023,141 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB6BE5C-06C9-4E21-B6D2-3A099BD83B31}">
-  <dimension ref="A1:DY9"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:DY7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.7109375" style="3" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" style="3" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="24.42578125" style="4" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="18.5703125" style="4" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="23.5703125" style="4" customWidth="1"/>
-    <col min="8" max="8" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.6640625" style="3" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="20.1640625" style="3" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="24.5" style="4" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5" style="4" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="23.5" style="4" customWidth="1"/>
+    <col min="8" max="8" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="35.5703125" style="4" customWidth="1"/>
-    <col min="17" max="17" width="22.85546875" style="4" customWidth="1"/>
-    <col min="18" max="18" width="21.28515625" style="4" customWidth="1"/>
-    <col min="19" max="19" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.28515625" style="4" customWidth="1"/>
-    <col min="23" max="23" width="12.5703125" style="4" customWidth="1"/>
-    <col min="24" max="24" width="18.28515625" style="4" customWidth="1"/>
-    <col min="25" max="25" width="20.85546875" style="4" customWidth="1"/>
-    <col min="26" max="26" width="18.5703125" style="4" customWidth="1"/>
-    <col min="27" max="27" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="35.5" style="4" customWidth="1"/>
+    <col min="17" max="17" width="22.83203125" style="4" customWidth="1"/>
+    <col min="18" max="18" width="21.33203125" style="4" customWidth="1"/>
+    <col min="19" max="19" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.33203125" style="4" customWidth="1"/>
+    <col min="23" max="23" width="12.5" style="4" customWidth="1"/>
+    <col min="24" max="24" width="18.33203125" style="4" customWidth="1"/>
+    <col min="25" max="25" width="20.83203125" style="4" customWidth="1"/>
+    <col min="26" max="26" width="18.5" style="4" customWidth="1"/>
+    <col min="27" max="27" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="14.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="22.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="12.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
     <col min="55" max="55" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="14.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="22.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="16.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="65" max="65" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="12.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
     <col min="75" max="75" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="14.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="22.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="16.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="85" max="85" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="12.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
     <col min="95" max="95" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="14.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="22.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="16.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="105" max="105" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="12.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
     <col min="115" max="115" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="14.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="22.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="16.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="125" max="125" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="126" max="126" width="12.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="129" max="129" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:129" ht="71.25">
+    <row r="1" spans="1:129" ht="76" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
         <v>12</v>
       </c>
@@ -8504,7 +8462,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:129" ht="78.75" customHeight="1">
+    <row r="2" spans="1:129" ht="78.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -8885,7 +8843,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:129" ht="18">
+    <row r="3" spans="1:129" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
@@ -9044,7 +9002,7 @@
       <c r="DX3" s="7"/>
       <c r="DY3" s="7"/>
     </row>
-    <row r="4" spans="1:129" ht="18">
+    <row r="4" spans="1:129" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -9433,7 +9391,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:129" ht="18">
+    <row r="5" spans="1:129" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -9822,7 +9780,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:129" ht="18">
+    <row r="6" spans="1:129" ht="18" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -10211,229 +10169,115 @@
         <v>209</v>
       </c>
     </row>
-    <row r="7" spans="1:129">
-      <c r="A7" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>212</v>
-      </c>
+    <row r="7" spans="1:129" x14ac:dyDescent="0.2">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
-      <c r="I7" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="J7" s="19" t="s">
-        <v>213</v>
-      </c>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
-      <c r="M7" s="3" t="s">
-        <v>214</v>
-      </c>
+      <c r="M7" s="3"/>
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
-      <c r="P7" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="Q7" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="R7" s="15">
-        <v>987654321</v>
-      </c>
-      <c r="S7" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="T7" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="U7" s="14" t="s">
-        <v>219</v>
-      </c>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
+      <c r="R7" s="15"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
+      <c r="U7" s="14"/>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
       <c r="Y7" s="3"/>
       <c r="Z7" s="3"/>
-      <c r="AA7" s="3">
-        <v>100</v>
-      </c>
-      <c r="AD7" s="19" t="s">
-        <v>213</v>
-      </c>
+      <c r="AD7" s="19"/>
       <c r="AE7" s="3"/>
       <c r="AF7" s="3"/>
-      <c r="AG7" s="16" t="s">
-        <v>214</v>
-      </c>
+      <c r="AG7" s="16"/>
       <c r="AH7" s="3"/>
       <c r="AI7" s="3"/>
-      <c r="AJ7" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="AK7" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="AL7" s="15">
-        <v>1234567890</v>
-      </c>
-      <c r="AM7" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="AN7" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="AO7" s="14" t="s">
-        <v>219</v>
-      </c>
+      <c r="AJ7" s="3"/>
+      <c r="AK7" s="3"/>
+      <c r="AL7" s="15"/>
+      <c r="AM7" s="3"/>
+      <c r="AN7" s="3"/>
+      <c r="AO7" s="14"/>
       <c r="AP7" s="3"/>
       <c r="AQ7" s="3"/>
       <c r="AR7" s="3"/>
       <c r="AS7" s="3"/>
       <c r="AT7" s="3"/>
-      <c r="AV7" s="3">
-        <v>0.52500000000000002</v>
-      </c>
-      <c r="AX7" s="19" t="s">
-        <v>213</v>
-      </c>
+      <c r="AX7" s="19"/>
       <c r="AY7" s="3"/>
       <c r="AZ7" s="3"/>
-      <c r="BA7" s="16" t="s">
-        <v>214</v>
-      </c>
+      <c r="BA7" s="16"/>
       <c r="BB7" s="3"/>
       <c r="BC7" s="3"/>
-      <c r="BD7" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="BE7" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="BF7" s="15">
-        <v>123123123</v>
-      </c>
-      <c r="BG7" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="BH7" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="BI7" s="13" t="s">
-        <v>225</v>
-      </c>
-      <c r="BP7" s="3">
-        <v>0.1075</v>
-      </c>
+      <c r="BD7" s="3"/>
+      <c r="BE7" s="3"/>
+      <c r="BF7" s="15"/>
+      <c r="BG7" s="3"/>
+      <c r="BH7" s="3"/>
+      <c r="BI7" s="13"/>
       <c r="BQ7" s="17"/>
-      <c r="BR7" s="19" t="s">
-        <v>213</v>
-      </c>
+      <c r="BR7" s="19"/>
       <c r="BS7" s="3"/>
       <c r="BT7" s="3"/>
-      <c r="BU7" s="16" t="s">
-        <v>214</v>
-      </c>
+      <c r="BU7" s="16"/>
       <c r="BV7" s="3"/>
       <c r="BW7" s="3"/>
       <c r="BX7" s="3"/>
       <c r="BY7" s="3"/>
-      <c r="BZ7" s="15">
-        <v>33333</v>
-      </c>
-      <c r="CA7" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="CB7" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="CC7" s="15" t="s">
-        <v>219</v>
-      </c>
+      <c r="BZ7" s="15"/>
+      <c r="CA7" s="3"/>
+      <c r="CB7" s="3"/>
+      <c r="CC7" s="15"/>
       <c r="CD7" s="3"/>
       <c r="CE7" s="3"/>
       <c r="CF7" s="3"/>
       <c r="CG7" s="3"/>
       <c r="CH7" s="3"/>
-      <c r="CI7" s="3">
-        <v>200</v>
-      </c>
       <c r="CK7" s="17"/>
-      <c r="CL7" s="19" t="s">
-        <v>213</v>
-      </c>
+      <c r="CL7" s="19"/>
       <c r="CM7" s="3"/>
       <c r="CN7" s="3"/>
-      <c r="CO7" s="3" t="s">
-        <v>214</v>
-      </c>
+      <c r="CO7" s="3"/>
       <c r="CP7" s="3"/>
       <c r="CQ7" s="3"/>
       <c r="CR7" s="3"/>
       <c r="CS7" s="3"/>
-      <c r="CT7" s="15">
-        <v>986475</v>
-      </c>
-      <c r="CU7" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="CV7" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="CW7" s="15" t="s">
-        <v>225</v>
-      </c>
+      <c r="CT7" s="15"/>
+      <c r="CU7" s="3"/>
+      <c r="CV7" s="3"/>
+      <c r="CW7" s="15"/>
       <c r="CX7" s="3"/>
       <c r="CY7" s="3"/>
       <c r="CZ7" s="3"/>
       <c r="DA7" s="3"/>
       <c r="DB7" s="3"/>
-      <c r="DC7" s="3">
-        <v>100</v>
-      </c>
       <c r="DE7" s="17"/>
-      <c r="DF7" s="19" t="s">
-        <v>213</v>
-      </c>
+      <c r="DF7" s="19"/>
       <c r="DG7" s="3"/>
       <c r="DH7" s="3"/>
-      <c r="DI7" s="3" t="s">
-        <v>214</v>
-      </c>
+      <c r="DI7" s="3"/>
       <c r="DJ7" s="3"/>
       <c r="DK7" s="3"/>
       <c r="DL7" s="3"/>
       <c r="DM7" s="3"/>
-      <c r="DN7" s="15">
-        <v>986475</v>
-      </c>
-      <c r="DO7" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="DP7" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="DQ7" s="15" t="s">
-        <v>225</v>
-      </c>
+      <c r="DN7" s="15"/>
+      <c r="DO7" s="3"/>
+      <c r="DP7" s="3"/>
+      <c r="DQ7" s="15"/>
       <c r="DR7" s="3"/>
       <c r="DS7" s="3"/>
       <c r="DT7" s="3"/>
       <c r="DU7" s="3"/>
       <c r="DV7" s="3"/>
-      <c r="DY7" s="17" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:129" ht="51" customHeight="1">
-      <c r="A9" s="18" t="s">
-        <v>226</v>
-      </c>
+      <c r="DY7" s="17"/>
     </row>
   </sheetData>
   <dataValidations count="9">
@@ -10473,43 +10317,43 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C07391C1-ADEA-4783-B088-82B2B03B51C1}">
-  <dimension ref="A1:W11"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:W10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="71.25">
+    <row r="1" spans="1:23" ht="73" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>20</v>
@@ -10558,7 +10402,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="65.25" customHeight="1">
+    <row r="2" spans="1:23" ht="65.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -10566,10 +10410,10 @@
         <v>32</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>36</v>
@@ -10620,21 +10464,21 @@
         <v>47</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="V2" s="5" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="18">
+    <row r="3" spans="1:23" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12" t="s">
@@ -10662,7 +10506,7 @@
       <c r="V3" s="7"/>
       <c r="W3" s="7"/>
     </row>
-    <row r="4" spans="1:23" ht="18">
+    <row r="4" spans="1:23" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -10733,7 +10577,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="18">
+    <row r="5" spans="1:23" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -10804,7 +10648,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="18">
+    <row r="6" spans="1:23" ht="18" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -10812,172 +10656,115 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="L6" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="M6" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="N6" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="O6" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="P6" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="Q6" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="R6" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="S6" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="T6" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="U6" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="V6" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="W6" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="O6" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="Q6" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="R6" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="S6" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="T6" s="7" t="s">
-        <v>251</v>
-      </c>
-      <c r="U6" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="V6" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="W6" s="7" t="s">
-        <v>254</v>
-      </c>
     </row>
-    <row r="7" spans="1:23">
-      <c r="A7" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>256</v>
-      </c>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="19"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="3" t="s">
-        <v>214</v>
-      </c>
+      <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
-      <c r="J7" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>258</v>
-      </c>
-      <c r="L7" s="15">
-        <v>987654321</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="O7" s="14" t="s">
-        <v>219</v>
-      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="14"/>
       <c r="P7" s="3"/>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
-      <c r="W7" s="3" t="b">
-        <v>1</v>
-      </c>
     </row>
-    <row r="8" spans="1:23">
-      <c r="A8" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>256</v>
-      </c>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="19"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
-      <c r="G8" s="3" t="s">
-        <v>214</v>
-      </c>
+      <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
-      <c r="J8" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>258</v>
-      </c>
-      <c r="L8" s="15">
-        <v>987654321</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="N8" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="O8" s="14" t="s">
-        <v>219</v>
-      </c>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="14"/>
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
       <c r="T8" s="3"/>
-      <c r="W8" s="3" t="b">
-        <v>1</v>
-      </c>
     </row>
-    <row r="10" spans="1:23" ht="20.25">
-      <c r="A10" s="18" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" ht="63" customHeight="1">
-      <c r="A11" s="18" t="s">
-        <v>261</v>
-      </c>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A10" s="18"/>
     </row>
   </sheetData>
   <dataValidations count="8">
@@ -11015,31 +10802,31 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43DC4B2E-DE37-4356-844D-2B6774F3300A}">
   <dimension ref="A1:L9"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.1640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.140625" customWidth="1"/>
-    <col min="11" max="11" width="22.140625" customWidth="1"/>
-    <col min="12" max="12" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.1640625" customWidth="1"/>
+    <col min="11" max="11" width="22.1640625" customWidth="1"/>
+    <col min="12" max="12" width="17.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="64.5">
+    <row r="1" spans="1:12" ht="61" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>262</v>
+        <v>247</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>20</v>
@@ -11069,7 +10856,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="18">
+    <row r="2" spans="1:12" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -11085,12 +10872,12 @@
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
     </row>
-    <row r="3" spans="1:12" ht="18">
+    <row r="3" spans="1:12" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12"/>
@@ -11103,7 +10890,7 @@
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
     </row>
-    <row r="4" spans="1:12" ht="18">
+    <row r="4" spans="1:12" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -11141,7 +10928,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="18">
+    <row r="5" spans="1:12" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -11179,7 +10966,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="18">
+    <row r="6" spans="1:12" ht="18" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -11187,60 +10974,60 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>264</v>
+        <v>249</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>265</v>
+        <v>250</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>266</v>
+        <v>251</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>267</v>
+        <v>252</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>269</v>
+        <v>254</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>270</v>
+        <v>255</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>273</v>
+        <v>258</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>210</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>274</v>
-      </c>
       <c r="D7" s="3" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>276</v>
+        <v>261</v>
       </c>
       <c r="I7" s="4">
         <v>271070801</v>
@@ -11251,30 +11038,30 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>210</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>276</v>
+        <v>261</v>
       </c>
       <c r="I8" s="4">
         <v>271070801</v>
@@ -11285,30 +11072,30 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>210</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>276</v>
+        <v>261</v>
       </c>
       <c r="I9" s="4">
         <v>271070801</v>
@@ -11342,29 +11129,29 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD03E25A-C84D-4D48-B73D-2E3BC0A89BB0}">
   <dimension ref="A1:J8"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="54">
+    <row r="1" spans="1:10" ht="61" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>20</v>
@@ -11388,7 +11175,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="18">
+    <row r="2" spans="1:10" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -11402,12 +11189,12 @@
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
     </row>
-    <row r="3" spans="1:10" ht="18">
+    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12"/>
@@ -11418,7 +11205,7 @@
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
     </row>
-    <row r="4" spans="1:10" ht="18">
+    <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -11450,7 +11237,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="18">
+    <row r="5" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -11482,7 +11269,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="18">
+    <row r="6" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -11490,89 +11277,89 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>280</v>
+        <v>265</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>281</v>
+        <v>266</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>282</v>
+        <v>267</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>283</v>
+        <v>268</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>284</v>
+        <v>269</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>285</v>
+        <v>270</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>286</v>
+        <v>271</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>210</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F7" s="15">
         <v>987654321</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J7" s="3" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>210</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F8" s="15">
         <v>987654321</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J8" s="3" t="b">
         <v>1</v>
@@ -11607,38 +11394,38 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BDF6E9F-389F-4489-BCEB-6DD5879DBE91}">
   <dimension ref="A1:AA7"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.140625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="75">
+    <row r="1" spans="1:27" ht="76" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
         <v>12</v>
       </c>
@@ -11721,12 +11508,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="60" customHeight="1">
+    <row r="2" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>289</v>
+        <v>274</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -11754,7 +11541,7 @@
       <c r="Z2" s="5"/>
       <c r="AA2" s="5"/>
     </row>
-    <row r="3" spans="1:27" ht="18">
+    <row r="3" spans="1:27" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
@@ -11799,7 +11586,7 @@
       <c r="Z3" s="7"/>
       <c r="AA3" s="7"/>
     </row>
-    <row r="4" spans="1:27" ht="18">
+    <row r="4" spans="1:27" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -11882,7 +11669,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="18">
+    <row r="5" spans="1:27" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -11965,7 +11752,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="18">
+    <row r="6" spans="1:27" ht="18" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -12048,66 +11835,66 @@
         <v>149</v>
       </c>
     </row>
-    <row r="7" spans="1:27">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>210</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>290</v>
+        <v>275</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="E7" s="15">
         <v>987654321</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="I7" s="3">
         <v>100</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="M7" s="15">
         <v>1234567890</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="P7" s="14" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="Q7" s="3">
         <v>100</v>
       </c>
       <c r="T7" s="16" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="U7" s="15">
         <v>123123123</v>
       </c>
       <c r="V7" s="3" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="X7" s="13" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="AA7" s="17" t="b">
         <v>1</v>
@@ -12143,45 +11930,45 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACD0C25A-DB46-45FD-AD1F-9D0E02F210FE}">
   <dimension ref="A1:DD9"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" style="4" customWidth="1"/>
-    <col min="4" max="4" width="25.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="25.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="17.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.6640625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:108" ht="75">
+    <row r="1" spans="1:108" ht="73" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>262</v>
+        <v>247</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>291</v>
+        <v>276</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>20</v>
@@ -12230,7 +12017,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:108" ht="18">
+    <row r="2" spans="1:108" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -12258,12 +12045,12 @@
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
     </row>
-    <row r="3" spans="1:108" ht="18">
+    <row r="3" spans="1:108" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12" t="s">
@@ -12292,7 +12079,7 @@
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
     </row>
-    <row r="4" spans="1:108" ht="18">
+    <row r="4" spans="1:108" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -12366,7 +12153,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:108" ht="18">
+    <row r="5" spans="1:108" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -12377,7 +12164,7 @@
         <v>77</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>292</v>
+        <v>277</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>77</v>
@@ -12440,7 +12227,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:108" ht="18">
+    <row r="6" spans="1:108" ht="18" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -12448,73 +12235,73 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>264</v>
+        <v>249</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>293</v>
+        <v>278</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>265</v>
+        <v>250</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>294</v>
+        <v>279</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>295</v>
+        <v>280</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>266</v>
+        <v>251</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>296</v>
+        <v>281</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>297</v>
+        <v>282</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>298</v>
+        <v>283</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>299</v>
+        <v>284</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>267</v>
+        <v>252</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>269</v>
+        <v>254</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>270</v>
+        <v>255</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>300</v>
+        <v>285</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>301</v>
+        <v>286</v>
       </c>
       <c r="S6" s="7" t="s">
-        <v>302</v>
+        <v>287</v>
       </c>
       <c r="T6" s="7" t="s">
-        <v>303</v>
+        <v>288</v>
       </c>
       <c r="U6" s="7" t="s">
-        <v>304</v>
+        <v>289</v>
       </c>
       <c r="V6" s="7" t="s">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="W6" s="7" t="s">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="X6" s="7" t="s">
-        <v>273</v>
+        <v>258</v>
       </c>
     </row>
-    <row r="7" spans="1:108">
+    <row r="7" spans="1:108" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>210</v>
       </c>
@@ -12522,27 +12309,27 @@
         <v>211</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>276</v>
+        <v>261</v>
       </c>
       <c r="P7" s="4">
         <v>271070801</v>
@@ -12635,35 +12422,35 @@
       <c r="DC7" s="3"/>
       <c r="DD7" s="3"/>
     </row>
-    <row r="8" spans="1:108">
+    <row r="8" spans="1:108" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>210</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>274</v>
-      </c>
       <c r="D8" s="4" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>276</v>
+        <v>261</v>
       </c>
       <c r="P8" s="4">
         <v>271070801</v>
@@ -12756,35 +12543,35 @@
       <c r="DC8" s="3"/>
       <c r="DD8" s="3"/>
     </row>
-    <row r="9" spans="1:108">
+    <row r="9" spans="1:108" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>210</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>276</v>
+        <v>261</v>
       </c>
       <c r="P9" s="4">
         <v>271070801</v>
@@ -12907,45 +12694,45 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{589C9B5C-2C65-468C-B018-503470942EE7}">
   <dimension ref="A1:X8"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" style="4" customWidth="1"/>
-    <col min="4" max="4" width="25.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="25.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="39.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.83203125" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="17.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.6640625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="75">
+    <row r="1" spans="1:24" ht="73" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>291</v>
+        <v>276</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>20</v>
@@ -12994,7 +12781,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="18">
+    <row r="2" spans="1:24" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>31</v>
       </c>
@@ -13022,12 +12809,12 @@
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
     </row>
-    <row r="3" spans="1:24" ht="18">
+    <row r="3" spans="1:24" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="12" t="s">
@@ -13056,7 +12843,7 @@
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
     </row>
-    <row r="4" spans="1:24" ht="18">
+    <row r="4" spans="1:24" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -13130,7 +12917,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="18">
+    <row r="5" spans="1:24" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
@@ -13141,7 +12928,7 @@
         <v>77</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>292</v>
+        <v>277</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>77</v>
@@ -13204,7 +12991,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:24" ht="18">
+    <row r="6" spans="1:24" ht="18" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
         <v>82</v>
       </c>
@@ -13212,73 +12999,73 @@
         <v>72</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>280</v>
+        <v>265</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>306</v>
+        <v>291</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>281</v>
+        <v>266</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>307</v>
+        <v>292</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>308</v>
+        <v>293</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>282</v>
+        <v>267</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>309</v>
+        <v>294</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>310</v>
+        <v>295</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>311</v>
+        <v>296</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>283</v>
+        <v>268</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>284</v>
+        <v>269</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>285</v>
+        <v>270</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>286</v>
+        <v>271</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>314</v>
+        <v>299</v>
       </c>
       <c r="S6" s="7" t="s">
-        <v>315</v>
+        <v>300</v>
       </c>
       <c r="T6" s="7" t="s">
-        <v>316</v>
+        <v>301</v>
       </c>
       <c r="U6" s="7" t="s">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="V6" s="7" t="s">
-        <v>318</v>
+        <v>303</v>
       </c>
       <c r="W6" s="7" t="s">
-        <v>319</v>
+        <v>304</v>
       </c>
       <c r="X6" s="7" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>210</v>
       </c>
@@ -13286,38 +13073,38 @@
         <v>211</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>321</v>
+        <v>306</v>
       </c>
       <c r="M7" s="15">
         <v>987654321</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="P7" s="14" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
@@ -13328,46 +13115,46 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>210</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="D8" s="3">
         <v>1</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>288</v>
+        <v>273</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="M8" s="15">
         <v>987654321</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="P8" s="14" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
@@ -13412,21 +13199,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d8c1821b-25b7-4bd3-913e-b4d27807b973" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Phase xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <Vertical xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <ProjectPhase xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <Owner xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <Comments xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <ContentDate xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
-    <Status xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04">Draft</Status>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -13702,22 +13480,57 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="d8c1821b-25b7-4bd3-913e-b4d27807b973" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Phase xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <Vertical xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <ProjectPhase xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <Owner xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <Comments xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <ContentDate xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04" xsi:nil="true"/>
+    <Status xmlns="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04">Draft</Status>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2289AEAC-15BB-46FC-8212-B4494D0EED04}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6241F7C5-31EE-4E6A-BD4F-9114CB87074C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95BEE76B-B7BD-4FAA-8DC3-5D013A61DA66}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{95BEE76B-B7BD-4FAA-8DC3-5D013A61DA66}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04"/>
+    <ds:schemaRef ds:uri="d8c1821b-25b7-4bd3-913e-b4d27807b973"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6241F7C5-31EE-4E6A-BD4F-9114CB87074C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2289AEAC-15BB-46FC-8212-B4494D0EED04}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d8c1821b-25b7-4bd3-913e-b4d27807b973"/>
+    <ds:schemaRef ds:uri="aeeb2937-3a82-4bf7-8e66-7d5cd46c6a04"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>